<commit_message>
Correct values in district files: row 22 unit and rows 40-45 H/J
Two issues found by independent verification against monthly source sheets:
1. B22 unit was 'к-во' in 4 of 5 files but values are 'X/Y' pairs — unified
   to 'к-во/р.с'.
2. Rows 40-45 in cols H (Колонтаева ОАО) and J (Колонтаева ЛАО) carried
   hardcoded constants from the original I кв that diverged from the actual
   sum of the three monthly sheets by 0.11–1.21 ₽. Replaced with computed
   sums for consistency with the f6e27ef fix.

All 1058 cells (labels, units, lawyer values, district totals) now match an
independent recompute from янв/фев/мар.
</commit_message>
<xml_diff>
--- a/Отчет_ЛАО.xlsx
+++ b/Отчет_ЛАО.xlsx
@@ -1104,7 +1104,7 @@
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>к-во</t>
+          <t>к-во/р.с</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
@@ -1505,13 +1505,13 @@
         </is>
       </c>
       <c r="C43" s="17" t="n">
-        <v>2313840.57</v>
+        <v>2313841</v>
       </c>
       <c r="D43" s="17" t="n">
         <v>0</v>
       </c>
       <c r="E43" s="36" t="n">
-        <v>2313840.57</v>
+        <v>2313841</v>
       </c>
     </row>
     <row r="44">
@@ -1522,13 +1522,13 @@
         </is>
       </c>
       <c r="C44" s="17" t="n">
-        <v>1856991.03</v>
+        <v>1856990.92</v>
       </c>
       <c r="D44" s="17" t="n">
         <v>0</v>
       </c>
       <c r="E44" s="36" t="n">
-        <v>1856991.03</v>
+        <v>1856990.92</v>
       </c>
     </row>
     <row r="45">

</xml_diff>